<commit_message>
Mejoras visuales: animaciones de carga, dialogos profesionales, iconos mejorados
</commit_message>
<xml_diff>
--- a/red_db.xlsx
+++ b/red_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -790,9 +790,13 @@
           <t>2026-03-02 11:24:05.067268</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>192.168.1.51</t>
+        </is>
+      </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -819,7 +823,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -856,7 +860,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -893,7 +897,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -901,9 +905,13 @@
           <t>2026-03-02 11:24:05.067268</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>192.168.1.217</t>
+        </is>
+      </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -930,7 +938,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -967,7 +975,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1004,7 +1012,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1041,7 +1049,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1078,7 +1086,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1115,7 +1123,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1152,7 +1160,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1189,7 +1197,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1226,7 +1234,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1263,7 +1271,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1300,7 +1308,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1337,7 +1345,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1374,7 +1382,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1411,7 +1419,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1448,7 +1456,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1485,7 +1493,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1522,7 +1530,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1559,7 +1567,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1596,7 +1604,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1633,7 +1641,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1670,7 +1678,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1707,7 +1715,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1744,7 +1752,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1781,7 +1789,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1818,7 +1826,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1855,7 +1863,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1892,7 +1900,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1929,7 +1937,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1937,9 +1945,13 @@
           <t>2026-03-02 11:24:05.067268</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>192.168.1.218</t>
+        </is>
+      </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I41" t="inlineStr"/>
     </row>
@@ -1966,7 +1978,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2003,7 +2015,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2040,7 +2052,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2077,7 +2089,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2109,12 +2121,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:34:15.418116</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2151,7 +2163,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2188,7 +2200,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2225,7 +2237,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2262,7 +2274,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2299,7 +2311,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2336,7 +2348,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2373,7 +2385,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2410,7 +2422,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2447,7 +2459,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2484,7 +2496,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2521,7 +2533,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2558,7 +2570,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2595,7 +2607,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2632,7 +2644,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2669,7 +2681,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2706,7 +2718,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2743,7 +2755,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2780,7 +2792,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2817,7 +2829,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2854,7 +2866,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2891,7 +2903,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2928,7 +2940,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2960,12 +2972,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:34:15.418116</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3002,7 +3014,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3039,7 +3051,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3076,7 +3088,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3113,7 +3125,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3150,7 +3162,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3187,7 +3199,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3224,7 +3236,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3256,12 +3268,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:34:15.418116</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3298,7 +3310,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3335,7 +3347,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3372,7 +3384,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3409,7 +3421,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3446,7 +3458,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3483,7 +3495,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3520,7 +3532,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3557,7 +3569,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2026-03-02 11:24:05.067268</t>
+          <t>2026-03-02 11:38:01.337230</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3570,6 +3582,1116 @@
         <v>0</v>
       </c>
       <c r="I85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>192.168.1.120</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>5E:EC:6B:5E:78:DC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:27:42.733001</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>192.168.1.126</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>02:B6:F1:0F:71:66</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:27:42.733001</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>192.168.1.199</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>3E:43:5A:6B:5E:70</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:27:42.733001</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>192.168.1.109</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>4E:8E:38:D6:66:25</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:34:15.418116</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>192.168.1.116</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>FE:11:5A:5C:22:1B</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:34:15.418116</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>192.168.1.147</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>52:DF:4F:AC:2E:43</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:34:15.418116</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>192.168.1.198</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>CE:A2:AE:CF:1F:12</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:34:15.418116</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>192.168.1.7</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>A2:3D:93:4A:31:41</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>192.168.1.3</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>192.168.1.6</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>192.168.1.13</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>192.168.1.17</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>192.168.1.18</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>192.168.1.23</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>192.168.1.27</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>192.168.1.31</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>192.168.1.38</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>192.168.1.41</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>192.168.1.45</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>192.168.1.49</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
+      <c r="I105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>192.168.1.68</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>192.168.1.64</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:36:39.826702</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>192.168.1.88</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>192.168.1.79</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>192.168.1.86</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>192.168.1.93</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>192.168.1.92</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>192.168.1.94</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>192.168.1.106</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
+      <c r="I114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>192.168.1.97</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>No detectada</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:38:01.337230</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>